<commit_message>
Streamlit demo setup - OCR project1
</commit_message>
<xml_diff>
--- a/data/reports/test_reports.xlsx
+++ b/data/reports/test_reports.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK7"/>
+  <dimension ref="A1:AK10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -616,20 +620,26 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>46014</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Liver Function Test (LFT)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Complete Blood Picture (CBP)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F2" t="n">
+        <v>416</v>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
@@ -641,50 +651,92 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>0.4</v>
+      </c>
       <c r="O2" t="n">
         <v>0.2</v>
       </c>
       <c r="P2" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="Q2" t="n">
+        <v>34</v>
+      </c>
+      <c r="R2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S2" t="n">
+        <v>219</v>
+      </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="X2" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
+      <c r="AG2" t="n">
+        <v>26</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>79</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>46012</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thyroid Test</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>Complete Blood Picture (CBP)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>416</v>
+      </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
@@ -696,44 +748,78 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>0.4</v>
+      </c>
       <c r="O3" t="n">
         <v>0.2</v>
       </c>
       <c r="P3" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="Q3" t="n">
+        <v>34</v>
+      </c>
+      <c r="R3" t="n">
+        <v>5</v>
+      </c>
+      <c r="S3" t="n">
+        <v>219</v>
+      </c>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="X3" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AG3" t="n">
+        <v>26</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>79</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>46010</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Complete Blood Picture (CBP)</t>
+          <t>Liver Function Test (LFT)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -781,14 +867,12 @@
       <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>46010</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Comprehensive Health Check</t>
+          <t>Thyroid Test</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -836,14 +920,12 @@
       <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>46010</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Liver Function Test (LFT)</t>
+          <t>Complete Blood Picture (CBP)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -891,28 +973,18 @@
       <c r="AK6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12-21</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>46010</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Complete Blood Picture (CBP)</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="D7" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="E7" t="n">
-        <v>10.54</v>
-      </c>
-      <c r="F7" t="n">
-        <v>416</v>
-      </c>
+          <t>Comprehensive Health Check</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
@@ -924,68 +996,279 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>0.4</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
         <v>0.2</v>
       </c>
       <c r="P7" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q7" t="n">
-        <v>34</v>
-      </c>
-      <c r="R7" t="n">
-        <v>5</v>
-      </c>
-      <c r="S7" t="n">
-        <v>219</v>
-      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="V7" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="W7" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="X7" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>78</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>32</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>12</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>8.199999999999999</v>
-      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="n">
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46010</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Liver Function Test (LFT)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>13</v>
+      </c>
+      <c r="J8" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>45908</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Complete Blood Picture (CBP)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E9" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F9" t="n">
+        <v>416</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>13</v>
+      </c>
+      <c r="J9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>34</v>
+      </c>
+      <c r="R9" t="n">
+        <v>5</v>
+      </c>
+      <c r="S9" t="n">
+        <v>219</v>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="X9" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="n">
         <v>26</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AH9" t="n">
         <v>79</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AI9" t="n">
         <v>2</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AJ9" t="n">
         <v>2</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="AK9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>45908</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Liver Function Test (LFT)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10.54</v>
+      </c>
+      <c r="F10" t="n">
+        <v>416</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>13</v>
+      </c>
+      <c r="J10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>34</v>
+      </c>
+      <c r="R10" t="n">
+        <v>5</v>
+      </c>
+      <c r="S10" t="n">
+        <v>219</v>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="X10" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="n">
+        <v>26</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>79</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK10" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>